<commit_message>
[PROGRAMMER] feat(audio): wire battle BGM trigger and The_Iron_Waltz asset (Plan34)
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoAudioEvents.xlsx
+++ b/Design/Data/ReEchoAudioEvents.xlsx
@@ -679,7 +679,11 @@
           <t>Music.Encounter</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Music/The_Iron_Waltz.The_Iron_Waltz</t>
+        </is>
+      </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
           <t>Music</t>

</xml_diff>

<commit_message>
[PROGRAMMER] complete Plan46 audio integration
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoAudioEvents.xlsx
+++ b/Design/Data/ReEchoAudioEvents.xlsx
@@ -627,7 +627,11 @@
           <t>Music.Menu</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Music/Music_Menu.Music_Menu</t>
+        </is>
+      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Music</t>
@@ -735,7 +739,11 @@
           <t>Music.Boss</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Music/Music_Boss.Music_Boss</t>
+        </is>
+      </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Music</t>
@@ -787,7 +795,11 @@
           <t>Music.Shop</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Music/Music_Shop.Music_Shop</t>
+        </is>
+      </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
           <t>Music</t>
@@ -839,7 +851,11 @@
           <t>Music.Death</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Music/Music_Death.Music_Death</t>
+        </is>
+      </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Music</t>
@@ -891,7 +907,11 @@
           <t>Music.Victory</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Music/Music_Victory.Music_Victory</t>
+        </is>
+      </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Music</t>
@@ -943,7 +963,11 @@
           <t>Ambience.Arena</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Ambience/Ambience_Arena.Ambience_Arena</t>
+        </is>
+      </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Ambience</t>
@@ -995,7 +1019,11 @@
           <t>Ambience.Rain</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Ambience/Ambience_Rain.Ambience_Rain</t>
+        </is>
+      </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Ambience</t>
@@ -1047,7 +1075,11 @@
           <t>UI.Hover</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/UI/UI_Hover.UI_Hover</t>
+        </is>
+      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
           <t>UiSfx</t>
@@ -1099,7 +1131,11 @@
           <t>UI.Confirm</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/UI/UI_Confirm.UI_Confirm</t>
+        </is>
+      </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
           <t>UiSfx</t>
@@ -1151,7 +1187,11 @@
           <t>UI.Cancel</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/UI/UI_Cancel.UI_Cancel</t>
+        </is>
+      </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
           <t>UiSfx</t>
@@ -1205,7 +1245,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>/Game/ReEcho/Audio/Diagnostics/ReEchoDiagTone.ReEchoDiagTone</t>
+          <t>/Game/ReEcho/Audio/UI/UI_Error.UI_Error</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1259,7 +1299,11 @@
           <t>UI.Purchase</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/UI/UI_Purchase.UI_Purchase</t>
+        </is>
+      </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
           <t>UiSfx</t>
@@ -1311,7 +1355,11 @@
           <t>UI.CardSelect</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/UI/UI_CardSelect.UI_CardSelect</t>
+        </is>
+      </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
           <t>UiSfx</t>
@@ -1363,7 +1411,11 @@
           <t>Combat.Attack</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Combat/Combat_Attack.Combat_Attack</t>
+        </is>
+      </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1415,7 +1467,11 @@
           <t>Combat.Hit</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Combat/Combat_Hit.Combat_Hit</t>
+        </is>
+      </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1467,7 +1523,11 @@
           <t>Combat.Block</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Combat/Combat_Block.Combat_Block</t>
+        </is>
+      </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1519,7 +1579,11 @@
           <t>Combat.Hurt</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Combat/Combat_Hurt.Combat_Hurt</t>
+        </is>
+      </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1571,7 +1635,11 @@
           <t>Combat.Kill</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Combat/Combat_Kill.Combat_Kill</t>
+        </is>
+      </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1623,7 +1691,11 @@
           <t>Combat.Death</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr"/>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Combat/Combat_Death.Combat_Death</t>
+        </is>
+      </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1675,7 +1747,11 @@
           <t>Enemy.Spawn</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr"/>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Enemy/Enemy_Spawn.Enemy_Spawn</t>
+        </is>
+      </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1727,7 +1803,11 @@
           <t>Enemy.Attack</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Enemy/Enemy_Attack.Enemy_Attack</t>
+        </is>
+      </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1779,7 +1859,11 @@
           <t>Enemy.Death</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Enemy/Enemy_Death.Enemy_Death</t>
+        </is>
+      </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1831,7 +1915,11 @@
           <t>Boss.Spawn</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Boss/Boss_Spawn.Boss_Spawn</t>
+        </is>
+      </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1883,7 +1971,11 @@
           <t>Boss.Attack</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Boss/Boss_Attack.Boss_Attack</t>
+        </is>
+      </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1935,7 +2027,11 @@
           <t>Boss.Death</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Boss/Boss_Death.Boss_Death</t>
+        </is>
+      </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -1987,7 +2083,11 @@
           <t>Echo.Spawn</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr"/>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Echo/Echo_Spawn.Echo_Spawn</t>
+        </is>
+      </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -2039,7 +2139,11 @@
           <t>Echo.Attack</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr"/>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Echo/Echo_Attack.Echo_Attack</t>
+        </is>
+      </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -2091,7 +2195,11 @@
           <t>Echo.End</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Echo/Echo_End.Echo_End</t>
+        </is>
+      </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
           <t>CombatSfx</t>
@@ -2143,7 +2251,11 @@
           <t>CameraMove</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Flow/CameraMove.CameraMove</t>
+        </is>
+      </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
           <t>UiSfx</t>
@@ -2195,7 +2307,11 @@
           <t>Revive</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr"/>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>/Game/ReEcho/Audio/Flow/Revive.Revive</t>
+        </is>
+      </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Music</t>

</xml_diff>

<commit_message>
[PROGRAMMER] sync canonical XLSX authoring workbooks to v1.1 production CSVs
The v1.1 commit e00ae185 shipped CSVs without updating Design/Data/ReEchoData.xlsx, so the authoring source stayed at v1.0 and validate_project.py failed the XLSX authoring sync gate.

- ReEchoData: add MinCardPackTier to tblCharacterAbilities; resync 11 tables (parts 111 rows, part_effects 129, card_effects 101, cards, characters, weapon_types, weapons, attack_steps, shop_price_ranges, shop_drop_levels)

- ReEchoEnemyData / ReEchoEncounterData / ReEchoAudioEvents: resync drifting tables (boss_phases, enemies, enemy_combat_stats, encounter_waves)

- restore embedded CR in multiline cells as &#13; (openpyxl strips CR on round-trip)

- normalise characters.csv to CRLF row terminators to match the generator
</commit_message>
<xml_diff>
--- a/Design/Data/ReEchoAudioEvents.xlsx
+++ b/Design/Data/ReEchoAudioEvents.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_ExportMap" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AudioEvents" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="_ExportMap" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="AudioEvents" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -527,12 +527,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P53"/>
+  <dimension ref="A1:R55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -657,10 +657,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F2" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -731,10 +729,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F3" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -813,10 +809,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F4" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -895,10 +889,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F5" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -977,10 +969,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F6" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -1055,10 +1045,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F7" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -1133,10 +1121,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F8" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -1207,10 +1193,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F9" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -1281,10 +1265,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F10" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -1355,10 +1337,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F11" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -1429,10 +1409,8 @@
           <t>Loop</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F12" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -1507,10 +1485,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F13" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -1585,10 +1561,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F14" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -1663,10 +1637,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F15" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
@@ -1713,8 +1685,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="P15" s="2" t="n">
-        <v>6.64</v>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>6.64</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -1739,10 +1713,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F16" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
@@ -1789,8 +1761,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="P16" s="2" t="n">
-        <v>6.64</v>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>6.64</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -1815,10 +1789,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F17" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
@@ -1893,10 +1865,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F18" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
@@ -1967,10 +1937,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F19" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
@@ -2049,10 +2017,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F20" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
@@ -2099,8 +2065,10 @@
           <t>2000</t>
         </is>
       </c>
-      <c r="P20" s="2" t="n">
-        <v>0.23</v>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>0.23</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -2129,10 +2097,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F21" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
@@ -2179,8 +2145,10 @@
           <t>2000</t>
         </is>
       </c>
-      <c r="P21" s="2" t="n">
-        <v>0.27</v>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>0.27</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -2209,10 +2177,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F22" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
@@ -2291,10 +2257,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F23" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
@@ -2341,8 +2305,10 @@
           <t>2000</t>
         </is>
       </c>
-      <c r="P23" s="2" t="n">
-        <v>1.36</v>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>1.36</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -2363,10 +2329,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F24" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
@@ -2445,10 +2409,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F25" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
@@ -2527,10 +2489,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F26" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
@@ -2577,8 +2537,10 @@
           <t>2000</t>
         </is>
       </c>
-      <c r="P26" s="2" t="n">
-        <v>0.42</v>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>0.42</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -2607,10 +2569,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F27" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
@@ -2689,10 +2649,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F28" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
@@ -2739,8 +2697,10 @@
           <t>2000</t>
         </is>
       </c>
-      <c r="P28" s="2" t="n">
-        <v>0.6</v>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>0.6</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -2761,10 +2721,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F29" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
@@ -2839,10 +2797,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F30" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
@@ -2889,8 +2845,10 @@
           <t>2000</t>
         </is>
       </c>
-      <c r="P30" s="2" t="n">
-        <v>0.93</v>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -2911,10 +2869,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F31" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
@@ -2989,10 +2945,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F32" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
@@ -3067,10 +3021,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F33" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
@@ -3141,10 +3093,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F34" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
@@ -3219,10 +3169,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F35" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
@@ -3293,10 +3241,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F36" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
@@ -3367,10 +3313,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F37" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
@@ -3445,10 +3389,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F38" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
@@ -3495,8 +3437,10 @@
           <t>2000</t>
         </is>
       </c>
-      <c r="P38" s="2" t="n">
-        <v>3.56</v>
+      <c r="P38" s="2" t="inlineStr">
+        <is>
+          <t>3.56</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -3517,10 +3461,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F39" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
@@ -3591,10 +3533,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F40" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
@@ -3665,10 +3605,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F41" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
@@ -3743,10 +3681,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F42" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -3821,10 +3757,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F43" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -3871,8 +3805,10 @@
           <t>0</t>
         </is>
       </c>
-      <c r="P43" s="2" t="n">
-        <v>6.64</v>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>6.64</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -3901,10 +3837,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F44" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
@@ -3983,10 +3917,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F45" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
@@ -4065,10 +3997,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F46" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
@@ -4147,10 +4077,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F47" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
@@ -4229,10 +4157,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F48" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
@@ -4307,10 +4233,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+      <c r="F49" s="2" t="b">
+        <v>1</v>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
@@ -4385,10 +4309,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F50" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
@@ -4463,10 +4385,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F51" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
@@ -4541,10 +4461,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F52" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
@@ -4619,10 +4537,8 @@
           <t>OneShot</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
+      <c r="F53" s="2" t="b">
+        <v>0</v>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
@@ -4669,12 +4585,20 @@
           <t>0</t>
         </is>
       </c>
-      <c r="P53" s="2" t="n">
-        <v>3.56</v>
-      </c>
-    </row>
+      <c r="P53" s="2" t="inlineStr">
+        <is>
+          <t>3.56</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
+    <row r="55"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="1" formatRows="1" sort="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
   <dataValidations count="4">
     <dataValidation sqref="D2:D53" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list" errorStyle="stop">
       <formula1>"Music,Ambience,CombatSfx,UiSfx"</formula1>
@@ -4689,9 +4613,5 @@
       <formula1>"PauseWithGame,ContinueOnPause"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
</xml_diff>